<commit_message>
more examples and updated research hours
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4FFC30A-3053-8644-816F-2F7660A7065F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F6FB449-E075-AA4A-A91A-10BF20915B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="740" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
+    <workbookView xWindow="1480" yWindow="740" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Date</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>worked on the hypothesis - U=M/C</t>
+  </si>
+  <si>
+    <t>continued working on more examples</t>
   </si>
 </sst>
 </file>
@@ -478,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="38.1640625" bestFit="1" customWidth="1"/>
@@ -512,8 +515,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C20)</f>
-        <v>16.66</v>
+        <f>SUM(C2:C21)</f>
+        <v>16.91</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -712,6 +715,17 @@
       </c>
       <c r="C20">
         <v>1.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>46080</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21">
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated research hours and examples from meeting
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F6FB449-E075-AA4A-A91A-10BF20915B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B56343A-98F7-ED4E-84B3-4A075105C7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="740" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t>Date</t>
   </si>
@@ -481,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="38.1640625" bestFit="1" customWidth="1"/>
@@ -515,8 +515,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C21)</f>
-        <v>16.91</v>
+        <f>SUM(C2:C22)</f>
+        <v>18.16</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -726,6 +726,17 @@
       </c>
       <c r="C21">
         <v>0.25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>46083</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>1.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated research hours again
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBC99908-4BC7-D249-A656-FEFD344F8924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{984E5230-3DF2-AA4A-84C4-B36E871C3899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="740" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -519,7 +519,7 @@
       </c>
       <c r="E2" s="3">
         <f>SUM(C2:C23)</f>
-        <v>19.16</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -750,7 +750,7 @@
         <v>20</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>1.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating research hours + new documents
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{984E5230-3DF2-AA4A-84C4-B36E871C3899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{87977764-2BE1-414E-B107-C799CF013BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="740" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
+    <workbookView xWindow="1460" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
   <si>
     <t>Date</t>
   </si>
@@ -99,14 +99,21 @@
   </si>
   <si>
     <t>worked on examples with decimals and infinities</t>
+  </si>
+  <si>
+    <t>continued testing examples/ going over presentation material</t>
+  </si>
+  <si>
+    <t>started working on I-Cat x I-Cat multiplication</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -144,12 +151,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,10 +492,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
   </cols>
@@ -518,8 +526,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C23)</f>
-        <v>19.41</v>
+        <f>SUM(C2:C26)</f>
+        <v>20.578999999999997</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -695,7 +703,7 @@
         <v>16</v>
       </c>
       <c r="C18">
-        <v>0.33</v>
+        <v>0.33300000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -751,6 +759,39 @@
       </c>
       <c r="C23">
         <v>1.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>46090</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24" s="5">
+        <v>0.33300000000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>46106</v>
+      </c>
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="2">
+        <v>46106</v>
+      </c>
+      <c r="B26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26" s="5">
+        <v>0.33300000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
draft of examples for presentation! (+ updated research hours)
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BCC9288-46D6-2C45-B964-A490F1A2078C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14699D5A-FB3C-9443-A8C2-CB44EA919F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t>started working on I-Cat x I-Cat multiplication</t>
+  </si>
+  <si>
+    <t>created examples for presentation</t>
   </si>
 </sst>
 </file>
@@ -492,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
@@ -526,8 +529,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C26)</f>
-        <v>20.745999999999999</v>
+        <f>SUM(C2:C27)</f>
+        <v>21.745999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -792,6 +795,17 @@
       </c>
       <c r="C26" s="4">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B27" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated research hours + presentation examples
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14699D5A-FB3C-9443-A8C2-CB44EA919F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEA11631-8C90-164C-B946-38D54C8BD6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>created examples for presentation</t>
+  </si>
+  <si>
+    <t>added more examples for presentation</t>
   </si>
 </sst>
 </file>
@@ -495,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
@@ -529,8 +532,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C27)</f>
-        <v>21.745999999999999</v>
+        <f>SUM(C2:C29)</f>
+        <v>22.995999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -806,6 +809,28 @@
       </c>
       <c r="C27">
         <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="2">
+        <v>46111</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="2">
+        <v>46112</v>
+      </c>
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29">
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
first draft of poster + updated hours
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8463070-62DF-3E4D-9F0E-B8ACB8554DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2ECD4DE-03CA-4F48-ACC7-E894AC3891FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1460" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
+    <workbookView xWindow="1440" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -114,6 +115,12 @@
   </si>
   <si>
     <t>presentation meeting</t>
+  </si>
+  <si>
+    <t>started creating poster</t>
+  </si>
+  <si>
+    <t>continued working on poster</t>
   </si>
 </sst>
 </file>
@@ -160,13 +167,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -501,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
@@ -535,8 +543,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C30)</f>
-        <v>23.995999999999999</v>
+        <f>SUM(C2:C32)</f>
+        <v>25.495999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -693,7 +701,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>46071</v>
       </c>
@@ -704,7 +712,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>46072</v>
       </c>
@@ -715,7 +723,7 @@
         <v>0.33300000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>46072</v>
       </c>
@@ -726,7 +734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>46079</v>
       </c>
@@ -737,7 +745,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>46080</v>
       </c>
@@ -748,7 +756,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>46083</v>
       </c>
@@ -759,7 +767,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>46090</v>
       </c>
@@ -770,7 +778,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>46090</v>
       </c>
@@ -781,7 +789,7 @@
         <v>0.33300000000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>46106</v>
       </c>
@@ -792,7 +800,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>46106</v>
       </c>
@@ -803,7 +811,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>46108</v>
       </c>
@@ -814,7 +822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>46111</v>
       </c>
@@ -825,7 +833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>46111</v>
       </c>
@@ -836,7 +844,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>46112</v>
       </c>
@@ -844,6 +852,29 @@
         <v>25</v>
       </c>
       <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="E30" s="6"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>46114</v>
+      </c>
+      <c r="B31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="2">
+        <v>46114</v>
+      </c>
+      <c r="B32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finished poster draft + updated hours
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2ECD4DE-03CA-4F48-ACC7-E894AC3891FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E828D99E-71F6-7F4E-A8E6-83E0FA9ADF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1440" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>continued working on poster</t>
+  </si>
+  <si>
+    <t>finished draft of poster + updated submission on website</t>
   </si>
 </sst>
 </file>
@@ -509,7 +512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
@@ -543,8 +546,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C32)</f>
-        <v>25.495999999999999</v>
+        <f>SUM(C2:C33)</f>
+        <v>26.245999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -875,7 +878,18 @@
         <v>27</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>46115</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished poster, updated presentation notebook, updated hours
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BEF27FD-B9DA-CB4B-A1D6-DC1B4F8A8450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A01BD01A-F407-3946-AA60-A93042B90B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1440" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>worked on poster</t>
+  </si>
+  <si>
+    <t>worked on I-Cat x I-Cat example</t>
+  </si>
+  <si>
+    <t>poster</t>
   </si>
 </sst>
 </file>
@@ -515,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
@@ -549,8 +555,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C36)</f>
-        <v>29.245999999999999</v>
+        <f>SUM(C2:C39)</f>
+        <v>34.995999999999995</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -926,6 +932,39 @@
       </c>
       <c r="C36">
         <v>1.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>46120</v>
+      </c>
+      <c r="B37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="2">
+        <v>46120</v>
+      </c>
+      <c r="B38" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="2">
+        <v>46120</v>
+      </c>
+      <c r="B39" t="s">
+        <v>31</v>
+      </c>
+      <c r="C39">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated research hours + poster
</commit_message>
<xml_diff>
--- a/AT/Research Hours.xlsx
+++ b/AT/Research Hours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abigailtouma/Desktop/SSS-Experiments/AT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A01BD01A-F407-3946-AA60-A93042B90B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5761414A-5CE2-8848-9BD5-5225D4569AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1440" yWindow="720" windowWidth="27640" windowHeight="16940" xr2:uid="{9D7B63EE-5957-9947-A3B5-024424A2FDD1}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
   <si>
     <t>Date</t>
   </si>
@@ -133,6 +132,27 @@
   </si>
   <si>
     <t>poster</t>
+  </si>
+  <si>
+    <t>final changes on poster</t>
+  </si>
+  <si>
+    <t>started working on presentation</t>
+  </si>
+  <si>
+    <t>worked on presentation outline</t>
+  </si>
+  <si>
+    <t>continued working on presentation</t>
+  </si>
+  <si>
+    <t>practiced presentation</t>
+  </si>
+  <si>
+    <t>research day!</t>
+  </si>
+  <si>
+    <t>physics presentation</t>
   </si>
 </sst>
 </file>
@@ -521,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542DF9F-5D83-964C-81A0-40C880F500E5}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="52.1640625" bestFit="1" customWidth="1"/>
@@ -555,8 +575,8 @@
         <v>1.25</v>
       </c>
       <c r="E2" s="3">
-        <f>SUM(C2:C39)</f>
-        <v>34.995999999999995</v>
+        <f>SUM(C2:C47)</f>
+        <v>41.412699999999994</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -965,6 +985,94 @@
       </c>
       <c r="C39">
         <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>46121</v>
+      </c>
+      <c r="B40" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>46124</v>
+      </c>
+      <c r="B41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="2">
+        <v>46125</v>
+      </c>
+      <c r="B42" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>46125</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="2">
+        <v>46126</v>
+      </c>
+      <c r="B44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="2">
+        <v>46127</v>
+      </c>
+      <c r="B45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="2">
+        <v>46128</v>
+      </c>
+      <c r="B46" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>46128</v>
+      </c>
+      <c r="B47" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47">
+        <v>0.16669999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>